<commit_message>
Alterada lógica de adição de personagens, perguntas atualizadas
</commit_message>
<xml_diff>
--- a/Dados_Iluminator.xlsx
+++ b/Dados_Iluminator.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO45"/>
+  <dimension ref="A1:BP50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -754,6 +754,11 @@
           <t>filhos</t>
         </is>
       </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>divulgação</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -777,7 +782,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>1.95</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
@@ -795,7 +800,7 @@
         <v>-1</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>1.95</v>
       </c>
       <c r="N2" t="n">
         <v>-1</v>
@@ -804,7 +809,7 @@
         <v>-1</v>
       </c>
       <c r="P2" t="n">
-        <v>1</v>
+        <v>1.75</v>
       </c>
       <c r="Q2" t="n">
         <v>1</v>
@@ -846,7 +851,7 @@
         <v>-1</v>
       </c>
       <c r="AD2" t="n">
-        <v>-1</v>
+        <v>-1.95</v>
       </c>
       <c r="AE2" t="n">
         <v>1</v>
@@ -864,7 +869,7 @@
         <v>-1</v>
       </c>
       <c r="AJ2" t="n">
-        <v>1</v>
+        <v>1.95</v>
       </c>
       <c r="AK2" t="n">
         <v>-1</v>
@@ -912,7 +917,7 @@
         <v>-1</v>
       </c>
       <c r="AZ2" t="n">
-        <v>-1</v>
+        <v>-1.95</v>
       </c>
       <c r="BA2" t="n">
         <v>-1</v>
@@ -948,7 +953,7 @@
         <v>1</v>
       </c>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>1.95</v>
       </c>
       <c r="BM2" t="n">
         <v>-1</v>
@@ -957,6 +962,9 @@
         <v>-1</v>
       </c>
       <c r="BO2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="BP2" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -1164,6 +1172,9 @@
       <c r="BO3" t="n">
         <v>1</v>
       </c>
+      <c r="BP3" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1369,6 +1380,9 @@
       <c r="BO4" t="n">
         <v>1</v>
       </c>
+      <c r="BP4" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1574,6 +1588,9 @@
       <c r="BO5" t="n">
         <v>-1</v>
       </c>
+      <c r="BP5" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1779,6 +1796,9 @@
       <c r="BO6" t="n">
         <v>-1</v>
       </c>
+      <c r="BP6" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1984,6 +2004,9 @@
       <c r="BO7" t="n">
         <v>-1</v>
       </c>
+      <c r="BP7" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2189,6 +2212,9 @@
       <c r="BO8" t="n">
         <v>-1</v>
       </c>
+      <c r="BP8" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2394,6 +2420,9 @@
       <c r="BO9" t="n">
         <v>-1</v>
       </c>
+      <c r="BP9" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2599,6 +2628,9 @@
       <c r="BO10" t="n">
         <v>1</v>
       </c>
+      <c r="BP10" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2804,6 +2836,9 @@
       <c r="BO11" t="n">
         <v>-1.95</v>
       </c>
+      <c r="BP11" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3009,6 +3044,9 @@
       <c r="BO12" t="n">
         <v>-1</v>
       </c>
+      <c r="BP12" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3214,6 +3252,9 @@
       <c r="BO13" t="n">
         <v>-1</v>
       </c>
+      <c r="BP13" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3419,6 +3460,9 @@
       <c r="BO14" t="n">
         <v>0</v>
       </c>
+      <c r="BP14" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3624,6 +3668,9 @@
       <c r="BO15" t="n">
         <v>-1</v>
       </c>
+      <c r="BP15" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3829,6 +3876,9 @@
       <c r="BO16" t="n">
         <v>-1</v>
       </c>
+      <c r="BP16" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4034,6 +4084,9 @@
       <c r="BO17" t="n">
         <v>-1</v>
       </c>
+      <c r="BP17" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4239,6 +4292,9 @@
       <c r="BO18" t="n">
         <v>-1</v>
       </c>
+      <c r="BP18" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4444,6 +4500,9 @@
       <c r="BO19" t="n">
         <v>-1</v>
       </c>
+      <c r="BP19" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4649,6 +4708,9 @@
       <c r="BO20" t="n">
         <v>-1</v>
       </c>
+      <c r="BP20" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4854,6 +4916,9 @@
       <c r="BO21" t="n">
         <v>-1</v>
       </c>
+      <c r="BP21" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5059,6 +5124,9 @@
       <c r="BO22" t="n">
         <v>-1</v>
       </c>
+      <c r="BP22" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5264,6 +5332,9 @@
       <c r="BO23" t="n">
         <v>-1</v>
       </c>
+      <c r="BP23" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5469,6 +5540,9 @@
       <c r="BO24" t="n">
         <v>-1</v>
       </c>
+      <c r="BP24" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5674,6 +5748,9 @@
       <c r="BO25" t="n">
         <v>-1</v>
       </c>
+      <c r="BP25" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5879,6 +5956,9 @@
       <c r="BO26" t="n">
         <v>0</v>
       </c>
+      <c r="BP26" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6084,6 +6164,9 @@
       <c r="BO27" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP27" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6289,6 +6372,9 @@
       <c r="BO28" t="n">
         <v>0</v>
       </c>
+      <c r="BP28" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6494,6 +6580,9 @@
       <c r="BO29" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP29" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6699,6 +6788,9 @@
       <c r="BO30" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP30" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6904,6 +6996,9 @@
       <c r="BO31" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP31" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7109,6 +7204,9 @@
       <c r="BO32" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP32" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7314,6 +7412,9 @@
       <c r="BO33" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP33" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7334,10 +7435,10 @@
         <v>-0.95</v>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>1.95</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.95</v>
+        <v>-1.9</v>
       </c>
       <c r="H34" t="n">
         <v>-2.85</v>
@@ -7358,7 +7459,7 @@
         <v>1.9</v>
       </c>
       <c r="N34" t="n">
-        <v>-0.95</v>
+        <v>-1.9</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
@@ -7418,13 +7519,13 @@
         <v>2.85</v>
       </c>
       <c r="AH34" t="n">
-        <v>-1.9</v>
+        <v>-2.85</v>
       </c>
       <c r="AI34" t="n">
         <v>-1</v>
       </c>
       <c r="AJ34" t="n">
-        <v>1.9</v>
+        <v>2.85</v>
       </c>
       <c r="AK34" t="n">
         <v>-1</v>
@@ -7518,6 +7619,9 @@
       </c>
       <c r="BO34" t="n">
         <v>-0.95</v>
+      </c>
+      <c r="BP34" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="35">
@@ -7724,6 +7828,9 @@
       <c r="BO35" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP35" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7759,7 +7866,7 @@
         <v>-0.95</v>
       </c>
       <c r="K36" t="n">
-        <v>-0.95</v>
+        <v>-1.9</v>
       </c>
       <c r="L36" t="n">
         <v>-0.95</v>
@@ -7768,7 +7875,7 @@
         <v>1.9</v>
       </c>
       <c r="N36" t="n">
-        <v>-1.9</v>
+        <v>-2.85</v>
       </c>
       <c r="O36" t="n">
         <v>-1</v>
@@ -7816,10 +7923,10 @@
         <v>-0.95</v>
       </c>
       <c r="AD36" t="n">
-        <v>3.8</v>
+        <v>4.75</v>
       </c>
       <c r="AE36" t="n">
-        <v>-1.9</v>
+        <v>-2.85</v>
       </c>
       <c r="AF36" t="n">
         <v>1</v>
@@ -7834,7 +7941,7 @@
         <v>1</v>
       </c>
       <c r="AJ36" t="n">
-        <v>-1.9</v>
+        <v>-2.85</v>
       </c>
       <c r="AK36" t="n">
         <v>1</v>
@@ -7867,7 +7974,7 @@
         <v>3.8</v>
       </c>
       <c r="AU36" t="n">
-        <v>1</v>
+        <v>1.75</v>
       </c>
       <c r="AV36" t="n">
         <v>1</v>
@@ -7928,6 +8035,9 @@
       </c>
       <c r="BO36" t="n">
         <v>-0.95</v>
+      </c>
+      <c r="BP36" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="37">
@@ -8134,6 +8244,9 @@
       <c r="BO37" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP37" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8339,6 +8452,9 @@
       <c r="BO38" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP38" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8544,6 +8660,9 @@
       <c r="BO39" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP39" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8749,6 +8868,9 @@
       <c r="BO40" t="n">
         <v>-0.95</v>
       </c>
+      <c r="BP40" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8778,19 +8900,19 @@
         <v>-0.95</v>
       </c>
       <c r="I41" t="n">
-        <v>1.9</v>
+        <v>2.85</v>
       </c>
       <c r="J41" t="n">
         <v>-0.95</v>
       </c>
       <c r="K41" t="n">
-        <v>-0.95</v>
+        <v>-1.9</v>
       </c>
       <c r="L41" t="n">
         <v>-0.95</v>
       </c>
       <c r="M41" t="n">
-        <v>1.9</v>
+        <v>0.95</v>
       </c>
       <c r="N41" t="n">
         <v>-1.9</v>
@@ -8802,13 +8924,13 @@
         <v>0.95</v>
       </c>
       <c r="Q41" t="n">
-        <v>-0.75</v>
+        <v>0.2</v>
       </c>
       <c r="R41" t="n">
         <v>0.75</v>
       </c>
       <c r="S41" t="n">
-        <v>-0.95</v>
+        <v>-1.9</v>
       </c>
       <c r="T41" t="n">
         <v>-0.95</v>
@@ -8817,7 +8939,7 @@
         <v>-0.95</v>
       </c>
       <c r="V41" t="n">
-        <v>-0.95</v>
+        <v>-1.9</v>
       </c>
       <c r="W41" t="n">
         <v>0.95</v>
@@ -8826,7 +8948,7 @@
         <v>-0.95</v>
       </c>
       <c r="Y41" t="n">
-        <v>0.95</v>
+        <v>1.9</v>
       </c>
       <c r="Z41" t="n">
         <v>-0.95</v>
@@ -8841,13 +8963,13 @@
         <v>-0.95</v>
       </c>
       <c r="AD41" t="n">
-        <v>0.95</v>
+        <v>0.2</v>
       </c>
       <c r="AE41" t="n">
         <v>-0.95</v>
       </c>
       <c r="AF41" t="n">
-        <v>-0.95</v>
+        <v>-1.9</v>
       </c>
       <c r="AG41" t="n">
         <v>-0.95</v>
@@ -8859,13 +8981,13 @@
         <v>0.95</v>
       </c>
       <c r="AJ41" t="n">
-        <v>-1.9</v>
+        <v>-2.85</v>
       </c>
       <c r="AK41" t="n">
         <v>-0.95</v>
       </c>
       <c r="AL41" t="n">
-        <v>0.95</v>
+        <v>1.9</v>
       </c>
       <c r="AM41" t="n">
         <v>-1</v>
@@ -8883,7 +9005,7 @@
         <v>-1</v>
       </c>
       <c r="AR41" t="n">
-        <v>-0.95</v>
+        <v>-1.9</v>
       </c>
       <c r="AS41" t="n">
         <v>1</v>
@@ -8898,7 +9020,7 @@
         <v>-0.95</v>
       </c>
       <c r="AW41" t="n">
-        <v>-0.95</v>
+        <v>-1.9</v>
       </c>
       <c r="AX41" t="n">
         <v>1</v>
@@ -8922,7 +9044,7 @@
         <v>-0.95</v>
       </c>
       <c r="BE41" t="n">
-        <v>-1</v>
+        <v>-1.95</v>
       </c>
       <c r="BF41" t="n">
         <v>-0.95</v>
@@ -8953,6 +9075,9 @@
       </c>
       <c r="BO41" t="n">
         <v>-0.95</v>
+      </c>
+      <c r="BP41" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="42">
@@ -9159,6 +9284,9 @@
       <c r="BO42" t="n">
         <v>-3</v>
       </c>
+      <c r="BP42" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -9364,6 +9492,9 @@
       <c r="BO43" t="n">
         <v>-3</v>
       </c>
+      <c r="BP43" t="n">
+        <v>-1</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -9396,7 +9527,7 @@
         <v>3</v>
       </c>
       <c r="J44" t="n">
-        <v>-3</v>
+        <v>-3.95</v>
       </c>
       <c r="K44" t="n">
         <v>-3</v>
@@ -9405,7 +9536,7 @@
         <v>-3</v>
       </c>
       <c r="M44" t="n">
-        <v>3.95</v>
+        <v>4.9</v>
       </c>
       <c r="N44" t="n">
         <v>3.95</v>
@@ -9420,7 +9551,7 @@
         <v>3</v>
       </c>
       <c r="R44" t="n">
-        <v>3.95</v>
+        <v>4.9</v>
       </c>
       <c r="S44" t="n">
         <v>3</v>
@@ -9468,7 +9599,7 @@
         <v>-3</v>
       </c>
       <c r="AH44" t="n">
-        <v>3</v>
+        <v>3.95</v>
       </c>
       <c r="AI44" t="n">
         <v>-3</v>
@@ -9501,7 +9632,7 @@
         <v>-3</v>
       </c>
       <c r="AS44" t="n">
-        <v>-3</v>
+        <v>-3.95</v>
       </c>
       <c r="AT44" t="n">
         <v>3</v>
@@ -9568,6 +9699,9 @@
       </c>
       <c r="BO44" t="n">
         <v>-3</v>
+      </c>
+      <c r="BP44" t="n">
+        <v>-1</v>
       </c>
     </row>
     <row r="45">
@@ -9772,6 +9906,1049 @@
         <v>-3</v>
       </c>
       <c r="BO45" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BP45" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Luiza (T25)</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="E46" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="I46" t="n">
+        <v>3</v>
+      </c>
+      <c r="J46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="K46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="L46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M46" t="n">
+        <v>3</v>
+      </c>
+      <c r="N46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="O46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>3</v>
+      </c>
+      <c r="R46" t="n">
+        <v>0</v>
+      </c>
+      <c r="S46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="T46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="U46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="V46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="W46" t="n">
+        <v>3</v>
+      </c>
+      <c r="X46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>-3.95</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>-3.95</v>
+      </c>
+      <c r="AB46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AD46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AE46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AF46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AG46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AH46" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="AI46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ46" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AL46" t="n">
+        <v>3</v>
+      </c>
+      <c r="AM46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AN46" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AP46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AQ46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AR46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AS46" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="AT46" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU46" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="AV46" t="n">
+        <v>3</v>
+      </c>
+      <c r="AW46" t="n">
+        <v>3</v>
+      </c>
+      <c r="AX46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AY46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AZ46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BA46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BB46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BC46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BD46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BE46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BF46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BG46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BH46" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="BI46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BJ46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BK46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BL46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BM46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BN46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BO46" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BP46" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Matheus Velloso (T25)</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="C47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="D47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="E47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="J47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="K47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="L47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="M47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="N47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="O47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="P47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="S47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="T47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="U47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="V47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="W47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="X47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AA47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AB47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AD47" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AE47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AF47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AG47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AI47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AJ47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AK47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AL47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AM47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AN47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AO47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AP47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AQ47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AR47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AS47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AT47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AU47" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="AV47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AW47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AX47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="AY47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="AZ47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="BA47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB47" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="BC47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BD47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BE47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="BF47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BG47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BH47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BI47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BJ47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BK47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BL47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BM47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BN47" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="BO47" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="BP47" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Caio Ketchup (T25)</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F48" t="n">
+        <v>3</v>
+      </c>
+      <c r="G48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="I48" t="n">
+        <v>3</v>
+      </c>
+      <c r="J48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="K48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="L48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M48" t="n">
+        <v>3</v>
+      </c>
+      <c r="N48" t="n">
+        <v>2</v>
+      </c>
+      <c r="O48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="P48" t="n">
+        <v>-2</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>3</v>
+      </c>
+      <c r="R48" t="n">
+        <v>-2</v>
+      </c>
+      <c r="S48" t="n">
+        <v>-2</v>
+      </c>
+      <c r="T48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="U48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="V48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="W48" t="n">
+        <v>3</v>
+      </c>
+      <c r="X48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AB48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AC48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AD48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AE48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AF48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AG48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AH48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AI48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AJ48" t="n">
+        <v>3</v>
+      </c>
+      <c r="AK48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AL48" t="n">
+        <v>2</v>
+      </c>
+      <c r="AM48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AN48" t="n">
+        <v>-2</v>
+      </c>
+      <c r="AO48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AP48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AQ48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AR48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AS48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AT48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AU48" t="n">
+        <v>-2</v>
+      </c>
+      <c r="AV48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AW48" t="n">
+        <v>3</v>
+      </c>
+      <c r="AX48" t="n">
+        <v>3</v>
+      </c>
+      <c r="AY48" t="n">
+        <v>2</v>
+      </c>
+      <c r="AZ48" t="n">
+        <v>-2</v>
+      </c>
+      <c r="BA48" t="n">
+        <v>-2</v>
+      </c>
+      <c r="BB48" t="n">
+        <v>-2</v>
+      </c>
+      <c r="BC48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BD48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BE48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BF48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BG48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BH48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BI48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BJ48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BK48" t="n">
+        <v>-2</v>
+      </c>
+      <c r="BL48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BM48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BN48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BO48" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BP48" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Aline (T25)</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>3</v>
+      </c>
+      <c r="C49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="G49" t="n">
+        <v>3</v>
+      </c>
+      <c r="H49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="I49" t="n">
+        <v>3</v>
+      </c>
+      <c r="J49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="K49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="L49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M49" t="n">
+        <v>3</v>
+      </c>
+      <c r="N49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="O49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="P49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>2</v>
+      </c>
+      <c r="R49" t="n">
+        <v>0</v>
+      </c>
+      <c r="S49" t="n">
+        <v>0</v>
+      </c>
+      <c r="T49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="U49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="V49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="W49" t="n">
+        <v>3</v>
+      </c>
+      <c r="X49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Y49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Z49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AA49" t="n">
+        <v>3</v>
+      </c>
+      <c r="AB49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AD49" t="n">
+        <v>3</v>
+      </c>
+      <c r="AE49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AF49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AG49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AH49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AI49" t="n">
+        <v>3</v>
+      </c>
+      <c r="AJ49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AK49" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AM49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AN49" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AP49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AQ49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AR49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AS49" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT49" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AV49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AW49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AX49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AY49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AZ49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BA49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BB49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BC49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BD49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BE49" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF49" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BH49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BI49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BJ49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BK49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BL49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BM49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BN49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BO49" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BP49" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Bruna (T25)</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>3</v>
+      </c>
+      <c r="C50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="E50" t="n">
+        <v>3</v>
+      </c>
+      <c r="F50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="G50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="I50" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="J50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="K50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="L50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="M50" t="n">
+        <v>3</v>
+      </c>
+      <c r="N50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="O50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="P50" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0</v>
+      </c>
+      <c r="R50" t="n">
+        <v>2</v>
+      </c>
+      <c r="S50" t="n">
+        <v>-2</v>
+      </c>
+      <c r="T50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="U50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="V50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="W50" t="n">
+        <v>3</v>
+      </c>
+      <c r="X50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="Z50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AA50" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="AB50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AC50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AD50" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AF50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AG50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AH50" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="AI50" t="n">
+        <v>3</v>
+      </c>
+      <c r="AJ50" t="n">
+        <v>-3.95</v>
+      </c>
+      <c r="AK50" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL50" t="n">
+        <v>-3.95</v>
+      </c>
+      <c r="AM50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AN50" t="n">
+        <v>3</v>
+      </c>
+      <c r="AO50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AP50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AQ50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AR50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AS50" t="n">
+        <v>3</v>
+      </c>
+      <c r="AT50" t="n">
+        <v>3</v>
+      </c>
+      <c r="AU50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AV50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AW50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AX50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AY50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="AZ50" t="n">
+        <v>-3.95</v>
+      </c>
+      <c r="BA50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BB50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BC50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BD50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BE50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BF50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BG50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BH50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BI50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BJ50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BK50" t="n">
+        <v>-2</v>
+      </c>
+      <c r="BL50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BM50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BN50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BO50" t="n">
+        <v>-3</v>
+      </c>
+      <c r="BP50" t="n">
         <v>-3</v>
       </c>
     </row>

</xml_diff>